<commit_message>
Polish public demo and add offline CI
</commit_message>
<xml_diff>
--- a/examples/output/part2_results.xlsx
+++ b/examples/output/part2_results.xlsx
@@ -889,7 +889,7 @@
       </c>
       <c r="AR2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T16:08:26+00:00</t>
+          <t>2026-10-17T08:47:00+00:00</t>
         </is>
       </c>
     </row>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="AI3" s="2" t="inlineStr">
         <is>
-          <t>["HTTP 200; ответ 211 байт; извлечено 45 символов.", "Проблемы извлечения: "]</t>
+          <t>["HTTP 200; ответ 211 байт; извлечено 45 символов."]</t>
         </is>
       </c>
       <c r="AJ3" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="AR3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T16:08:26+00:00</t>
+          <t>2026-10-17T08:47:00+00:00</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="AR4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T16:08:26+00:00</t>
+          <t>2026-10-17T08:47:00+00:00</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1459,7 @@
       </c>
       <c r="AR5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T16:08:26+00:00</t>
+          <t>2026-10-17T08:47:00+00:00</t>
         </is>
       </c>
     </row>
@@ -1645,7 +1645,7 @@
       </c>
       <c r="AR6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T16:08:26+00:00</t>
+          <t>2026-10-17T08:47:00+00:00</t>
         </is>
       </c>
     </row>
@@ -1841,7 +1841,7 @@
       </c>
       <c r="AR7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T16:08:26+00:00</t>
+          <t>2026-10-17T08:47:00+00:00</t>
         </is>
       </c>
     </row>
@@ -2023,7 +2023,7 @@
       </c>
       <c r="AR8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T16:08:26+00:00</t>
+          <t>2026-10-17T08:47:00+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Polish Excel rights-holder header and documentation
</commit_message>
<xml_diff>
--- a/examples/output/part2_results.xlsx
+++ b/examples/output/part2_results.xlsx
@@ -893,7 +893,7 @@
       </c>
       <c r="AR2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T17:31:45+00:00</t>
+          <t>2026-10-31T11:45:15+00:00</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="AR3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T17:31:45+00:00</t>
+          <t>2026-10-31T11:45:15+00:00</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="AR4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T17:31:45+00:00</t>
+          <t>2026-10-31T11:45:15+00:00</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="AR5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T17:31:45+00:00</t>
+          <t>2026-10-31T11:45:15+00:00</t>
         </is>
       </c>
     </row>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="AR6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T17:31:45+00:00</t>
+          <t>2026-10-31T11:45:15+00:00</t>
         </is>
       </c>
     </row>
@@ -1843,7 +1843,7 @@
       </c>
       <c r="AR7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T17:31:45+00:00</t>
+          <t>2026-10-31T11:45:15+00:00</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="AR8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T17:31:45+00:00</t>
+          <t>2026-10-31T11:45:15+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>